<commit_message>
Add lead schema, Excel lead/project import and lead research (v1)
</commit_message>
<xml_diff>
--- a/backend/scripts/sample_leads.xlsx
+++ b/backend/scripts/sample_leads.xlsx
@@ -417,21 +417,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -562,7 +562,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Python Software Foundation</t>
+          <t>PetMD</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -577,17 +577,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>python.org</t>
+          <t>petmd.com</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Non-profit Organizations</t>
+          <t>Veterinary Services</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>11-50 employees</t>
+          <t>51-200 employees</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -610,7 +610,11 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Pet health records assistant</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -620,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mozilla Foundation</t>
+          <t>Tire Rack</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -631,17 +635,17 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://www.mozilla.org</t>
+          <t>https://www.tirerack.com</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Software Development</t>
+          <t>Retail Motor Vehicles</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>201-500 employees</t>
+          <t>501-1,000 employees</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -674,7 +678,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Wikimedia Foundation</t>
+          <t>Flexport</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -685,17 +689,17 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>wikimediafoundation.org</t>
+          <t>flexport.com</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Non-profit Organizations</t>
+          <t>Transportation, Logistics, Supply Chain and Storage</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>501-1,000 employees</t>
+          <t>1,001-5,000 employees</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -728,7 +732,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Django Software Foundation</t>
+          <t>Scholarship America</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -739,17 +743,17 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>djangoproject.com</t>
+          <t>scholarshipamerica.org</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Software Development</t>
+          <t>Non-profit Organizations</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1-10 employees</t>
+          <t>51-200 employees</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -774,7 +778,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Web platform rebuild</t>
+          <t>Scholarship application platform</t>
         </is>
       </c>
     </row>
@@ -786,7 +790,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mystery Logistics Pvt Ltd</t>
+          <t>Harbor Table Restaurants Pvt Ltd</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -798,7 +802,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Transportation, Logistics, Supply Chain</t>
+          <t>Restaurants</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -826,7 +830,11 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Menu recommendation app for diners</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -836,7 +844,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Python Software Foundation</t>
+          <t>PetMD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -848,7 +856,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Non-profit Organizations</t>
+          <t>Veterinary Services</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -856,7 +864,11 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Pet health records assistant</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1015,6 +1027,176 @@
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Rahul Menon</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Atlassian</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>+1 212 555 0109</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.atlassian.com</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Software Development</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>5,001-10,000 employees</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Linkedin-Sales</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Internal knowledge chatbot</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Elena Petrova</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CrowdStrike</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>+1 212 555 0110</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>crowdstrike.com</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Computer and Network Security</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>5,001-10,000 employees</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Cold Email</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Security analyst assistant</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Jordan Blake</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>OpenTable</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>+1 212 555 0111</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>opentable.com</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Restaurants</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1,001-5,000 employees</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Linkedin-Sales</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>